<commit_message>
fixed algorithms and solver and reran experiments
</commit_message>
<xml_diff>
--- a/Experiments/outputs/scenario_1.xlsx
+++ b/Experiments/outputs/scenario_1.xlsx
@@ -530,55 +530,55 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>571.5363917066093</v>
+        <v>543.7061298606694</v>
       </c>
       <c r="D2" t="n">
-        <v>0.201469898223877</v>
+        <v>0.7176141738891602</v>
       </c>
       <c r="E2" t="n">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F2" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G2" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="H2" t="n">
-        <v>1150.636200185768</v>
+        <v>1220.910916354952</v>
       </c>
       <c r="I2" t="n">
-        <v>0.8132452964782715</v>
+        <v>4.659343004226685</v>
       </c>
       <c r="J2" t="n">
-        <v>222</v>
+        <v>253</v>
       </c>
       <c r="K2" t="n">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="L2" t="n">
-        <v>255</v>
+        <v>332</v>
       </c>
       <c r="M2" t="n">
-        <v>3753.772218132347</v>
+        <v>3694.350564602827</v>
       </c>
       <c r="N2" t="n">
-        <v>5.407880067825317</v>
+        <v>4.762768745422363</v>
       </c>
       <c r="O2" t="n">
-        <v>1142</v>
+        <v>1283</v>
       </c>
       <c r="P2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>3825</v>
+        <v>4333</v>
       </c>
       <c r="R2" t="n">
-        <v>0.8477434541856746</v>
+        <v>0.8528276836881281</v>
       </c>
       <c r="S2" t="n">
-        <v>0.6934720240541776</v>
+        <v>0.669519474396115</v>
       </c>
     </row>
     <row r="3">
@@ -591,55 +591,55 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>630.2502078711502</v>
+        <v>586.2974412235982</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2221581935882568</v>
+        <v>0.3080582618713379</v>
       </c>
       <c r="E3" t="n">
-        <v>174</v>
+        <v>153</v>
       </c>
       <c r="F3" t="n">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="G3" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="H3" t="n">
-        <v>1257.824054704108</v>
+        <v>1328.097787713385</v>
       </c>
       <c r="I3" t="n">
-        <v>0.7781009674072266</v>
+        <v>4.720230102539062</v>
       </c>
       <c r="J3" t="n">
-        <v>207</v>
+        <v>244</v>
       </c>
       <c r="K3" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="L3" t="n">
-        <v>245</v>
+        <v>328</v>
       </c>
       <c r="M3" t="n">
-        <v>3849.486008831443</v>
+        <v>3740.304788587463</v>
       </c>
       <c r="N3" t="n">
-        <v>5.458893060684204</v>
+        <v>5.031516075134277</v>
       </c>
       <c r="O3" t="n">
-        <v>1156</v>
+        <v>1311</v>
       </c>
       <c r="P3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>3811</v>
+        <v>4385</v>
       </c>
       <c r="R3" t="n">
-        <v>0.8362767895700263</v>
+        <v>0.8432487526116782</v>
       </c>
       <c r="S3" t="n">
-        <v>0.6732488306702703</v>
+        <v>0.6449225764259323</v>
       </c>
     </row>
     <row r="4">
@@ -652,55 +652,55 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>587.18374438052</v>
+        <v>635.2291820965082</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2587668895721436</v>
+        <v>0.3377640247344971</v>
       </c>
       <c r="E4" t="n">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="F4" t="n">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="G4" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="H4" t="n">
-        <v>1217.494640956626</v>
+        <v>1193.868177324222</v>
       </c>
       <c r="I4" t="n">
-        <v>0.6837120056152344</v>
+        <v>4.372910022735596</v>
       </c>
       <c r="J4" t="n">
-        <v>205</v>
+        <v>235</v>
       </c>
       <c r="K4" t="n">
         <v>33</v>
       </c>
       <c r="L4" t="n">
-        <v>237</v>
+        <v>310</v>
       </c>
       <c r="M4" t="n">
-        <v>3760.602202004754</v>
+        <v>3566.536547893981</v>
       </c>
       <c r="N4" t="n">
-        <v>6.775984048843384</v>
+        <v>5.29403281211853</v>
       </c>
       <c r="O4" t="n">
-        <v>1127</v>
+        <v>1283</v>
       </c>
       <c r="P4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>3661</v>
+        <v>4349</v>
       </c>
       <c r="R4" t="n">
-        <v>0.8438591180775525</v>
+        <v>0.8218918624367925</v>
       </c>
       <c r="S4" t="n">
-        <v>0.676250085609271</v>
+        <v>0.665258392479058</v>
       </c>
     </row>
     <row r="5">
@@ -713,55 +713,55 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>655.7753639500837</v>
+        <v>553.3327473177253</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2339928150177002</v>
+        <v>0.3350279331207275</v>
       </c>
       <c r="E5" t="n">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="F5" t="n">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="G5" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="H5" t="n">
-        <v>1288.482015950435</v>
+        <v>1337.368056240483</v>
       </c>
       <c r="I5" t="n">
-        <v>0.8829548358917236</v>
+        <v>4.685481071472168</v>
       </c>
       <c r="J5" t="n">
-        <v>231</v>
+        <v>240</v>
       </c>
       <c r="K5" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="L5" t="n">
-        <v>265</v>
+        <v>333</v>
       </c>
       <c r="M5" t="n">
-        <v>3758.606434309909</v>
+        <v>3824.411710957298</v>
       </c>
       <c r="N5" t="n">
-        <v>4.457988023757935</v>
+        <v>4.906610012054443</v>
       </c>
       <c r="O5" t="n">
-        <v>1134</v>
+        <v>1307</v>
       </c>
       <c r="P5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q5" t="n">
-        <v>3696</v>
+        <v>4348</v>
       </c>
       <c r="R5" t="n">
-        <v>0.8255269937379102</v>
+        <v>0.8553155912235142</v>
       </c>
       <c r="S5" t="n">
-        <v>0.6571915579698079</v>
+        <v>0.6503075094115003</v>
       </c>
     </row>
     <row r="6">
@@ -774,55 +774,55 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>515.0999298629116</v>
+        <v>629.4080914323436</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1862328052520752</v>
+        <v>0.3616702556610107</v>
       </c>
       <c r="E6" t="n">
-        <v>179</v>
+        <v>156</v>
       </c>
       <c r="F6" t="n">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="G6" t="n">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="H6" t="n">
-        <v>1184.214458979334</v>
+        <v>1195.825186770982</v>
       </c>
       <c r="I6" t="n">
-        <v>0.6515350341796875</v>
+        <v>3.486193895339966</v>
       </c>
       <c r="J6" t="n">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="K6" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="L6" t="n">
-        <v>247</v>
+        <v>285</v>
       </c>
       <c r="M6" t="n">
-        <v>3745.915794344307</v>
+        <v>3719.587133424859</v>
       </c>
       <c r="N6" t="n">
-        <v>5.24445915222168</v>
+        <v>5.006779909133911</v>
       </c>
       <c r="O6" t="n">
-        <v>1124</v>
+        <v>1241</v>
       </c>
       <c r="P6" t="n">
         <v>2</v>
       </c>
       <c r="Q6" t="n">
-        <v>3638</v>
+        <v>4069</v>
       </c>
       <c r="R6" t="n">
-        <v>0.8624902538811404</v>
+        <v>0.8307854961169285</v>
       </c>
       <c r="S6" t="n">
-        <v>0.6838651683608864</v>
+        <v>0.6785059352353684</v>
       </c>
     </row>
     <row r="7">
@@ -835,55 +835,55 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>619.1577601899488</v>
+        <v>565.1855150041837</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2448849678039551</v>
+        <v>0.3434789180755615</v>
       </c>
       <c r="E7" t="n">
-        <v>149</v>
+        <v>170</v>
       </c>
       <c r="F7" t="n">
+        <v>30</v>
+      </c>
+      <c r="G7" t="n">
+        <v>28</v>
+      </c>
+      <c r="H7" t="n">
+        <v>1285.673997673512</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4.004194974899292</v>
+      </c>
+      <c r="J7" t="n">
+        <v>218</v>
+      </c>
+      <c r="K7" t="n">
         <v>35</v>
       </c>
-      <c r="G7" t="n">
-        <v>26</v>
-      </c>
-      <c r="H7" t="n">
-        <v>1245.237091227444</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.6907346248626709</v>
-      </c>
-      <c r="J7" t="n">
-        <v>197</v>
-      </c>
-      <c r="K7" t="n">
-        <v>45</v>
-      </c>
       <c r="L7" t="n">
-        <v>241</v>
+        <v>306</v>
       </c>
       <c r="M7" t="n">
-        <v>3706.69288721257</v>
+        <v>3785.636035103777</v>
       </c>
       <c r="N7" t="n">
-        <v>4.557116270065308</v>
+        <v>6.561731100082397</v>
       </c>
       <c r="O7" t="n">
-        <v>1153</v>
+        <v>1299</v>
       </c>
       <c r="P7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>3734</v>
+        <v>4399</v>
       </c>
       <c r="R7" t="n">
-        <v>0.8329622175265901</v>
+        <v>0.8507026270451564</v>
       </c>
       <c r="S7" t="n">
-        <v>0.6640571179977467</v>
+        <v>0.6603809806987249</v>
       </c>
     </row>
     <row r="8">
@@ -896,55 +896,55 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>554.4600586629681</v>
+        <v>528.5340978071745</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2254910469055176</v>
+        <v>0.3735013008117676</v>
       </c>
       <c r="E8" t="n">
-        <v>173</v>
+        <v>197</v>
       </c>
       <c r="F8" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="G8" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="H8" t="n">
-        <v>1265.640353911451</v>
+        <v>1236.006655950854</v>
       </c>
       <c r="I8" t="n">
-        <v>0.867973804473877</v>
+        <v>5.334710121154785</v>
       </c>
       <c r="J8" t="n">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="K8" t="n">
         <v>36</v>
       </c>
       <c r="L8" t="n">
-        <v>266</v>
+        <v>307</v>
       </c>
       <c r="M8" t="n">
-        <v>3821.558002508315</v>
+        <v>3688.069915028062</v>
       </c>
       <c r="N8" t="n">
-        <v>4.656294107437134</v>
+        <v>5.959676742553711</v>
       </c>
       <c r="O8" t="n">
-        <v>1140</v>
+        <v>1312</v>
       </c>
       <c r="P8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q8" t="n">
-        <v>3730</v>
+        <v>4320</v>
       </c>
       <c r="R8" t="n">
-        <v>0.8549125622850567</v>
+        <v>0.8566908681276578</v>
       </c>
       <c r="S8" t="n">
-        <v>0.6688156105230547</v>
+        <v>0.6648635507384493</v>
       </c>
     </row>
     <row r="9">
@@ -957,55 +957,55 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>569.7988446803886</v>
+        <v>555.1987528523355</v>
       </c>
       <c r="D9" t="n">
-        <v>0.2011919021606445</v>
+        <v>0.4874527454376221</v>
       </c>
       <c r="E9" t="n">
-        <v>194</v>
+        <v>162</v>
       </c>
       <c r="F9" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G9" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="H9" t="n">
-        <v>1209.614789973352</v>
+        <v>1194.964106960657</v>
       </c>
       <c r="I9" t="n">
-        <v>0.7083590030670166</v>
+        <v>5.353314161300659</v>
       </c>
       <c r="J9" t="n">
-        <v>238</v>
+        <v>209</v>
       </c>
       <c r="K9" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="L9" t="n">
-        <v>266</v>
+        <v>288</v>
       </c>
       <c r="M9" t="n">
-        <v>3826.407624691334</v>
+        <v>3717.314433596681</v>
       </c>
       <c r="N9" t="n">
-        <v>4.785193920135498</v>
+        <v>5.793797016143799</v>
       </c>
       <c r="O9" t="n">
-        <v>1174</v>
+        <v>1238</v>
       </c>
       <c r="P9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>3973</v>
+        <v>4157</v>
       </c>
       <c r="R9" t="n">
-        <v>0.8510877824402326</v>
+        <v>0.8506452002460405</v>
       </c>
       <c r="S9" t="n">
-        <v>0.6838771744631029</v>
+        <v>0.678541019785493</v>
       </c>
     </row>
     <row r="10">
@@ -1018,55 +1018,55 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>581.7762853153192</v>
+        <v>567.2010701443188</v>
       </c>
       <c r="D10" t="n">
-        <v>0.2126750946044922</v>
+        <v>0.6813888549804688</v>
       </c>
       <c r="E10" t="n">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="F10" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="G10" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H10" t="n">
-        <v>1228.216713881184</v>
+        <v>1206.230723230933</v>
       </c>
       <c r="I10" t="n">
-        <v>0.8341660499572754</v>
+        <v>5.646857023239136</v>
       </c>
       <c r="J10" t="n">
-        <v>222</v>
+        <v>208</v>
       </c>
       <c r="K10" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="L10" t="n">
-        <v>261</v>
+        <v>293</v>
       </c>
       <c r="M10" t="n">
-        <v>3816.646245187828</v>
+        <v>3732.29123166143</v>
       </c>
       <c r="N10" t="n">
-        <v>4.363404989242554</v>
+        <v>6.639791965484619</v>
       </c>
       <c r="O10" t="n">
-        <v>1119</v>
+        <v>1325</v>
       </c>
       <c r="P10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q10" t="n">
-        <v>3769</v>
+        <v>4445</v>
       </c>
       <c r="R10" t="n">
-        <v>0.8475687166320838</v>
+        <v>0.8480287215175786</v>
       </c>
       <c r="S10" t="n">
-        <v>0.6781947723266818</v>
+        <v>0.6768122720439533</v>
       </c>
     </row>
     <row r="11">
@@ -1079,55 +1079,55 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>555.8992949299468</v>
+        <v>524.6696420168191</v>
       </c>
       <c r="D11" t="n">
-        <v>0.1816201210021973</v>
+        <v>0.4924421310424805</v>
       </c>
       <c r="E11" t="n">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="F11" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G11" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H11" t="n">
-        <v>1209.473226999412</v>
+        <v>1352.600099826511</v>
       </c>
       <c r="I11" t="n">
-        <v>0.6296501159667969</v>
+        <v>6.284840822219849</v>
       </c>
       <c r="J11" t="n">
-        <v>196</v>
+        <v>235</v>
       </c>
       <c r="K11" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="L11" t="n">
-        <v>231</v>
+        <v>322</v>
       </c>
       <c r="M11" t="n">
-        <v>3821.534879598427</v>
+        <v>3676.835729304653</v>
       </c>
       <c r="N11" t="n">
-        <v>5.059240818023682</v>
+        <v>6.213030815124512</v>
       </c>
       <c r="O11" t="n">
-        <v>1157</v>
+        <v>1237</v>
       </c>
       <c r="P11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q11" t="n">
-        <v>3800</v>
+        <v>4065</v>
       </c>
       <c r="R11" t="n">
-        <v>0.8545350723088621</v>
+        <v>0.8573040297027242</v>
       </c>
       <c r="S11" t="n">
-        <v>0.6835111375127616</v>
+        <v>0.6321293091648922</v>
       </c>
     </row>
     <row r="12">
@@ -1140,55 +1140,55 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>633.5922477345399</v>
+        <v>582.8598490369245</v>
       </c>
       <c r="D12" t="n">
-        <v>0.2165260314941406</v>
+        <v>0.5198209285736084</v>
       </c>
       <c r="E12" t="n">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="F12" t="n">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="G12" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="H12" t="n">
-        <v>1322.198394167079</v>
+        <v>1287.109095627238</v>
       </c>
       <c r="I12" t="n">
-        <v>0.7461497783660889</v>
+        <v>5.642041683197021</v>
       </c>
       <c r="J12" t="n">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="K12" t="n">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="L12" t="n">
-        <v>260</v>
+        <v>308</v>
       </c>
       <c r="M12" t="n">
-        <v>3805.853767733428</v>
+        <v>3705.186227970281</v>
       </c>
       <c r="N12" t="n">
-        <v>5.548770904541016</v>
+        <v>5.699030160903931</v>
       </c>
       <c r="O12" t="n">
-        <v>1128</v>
+        <v>1258</v>
       </c>
       <c r="P12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q12" t="n">
-        <v>3802</v>
+        <v>4112</v>
       </c>
       <c r="R12" t="n">
-        <v>0.8335216520649781</v>
+        <v>0.8426908087272531</v>
       </c>
       <c r="S12" t="n">
-        <v>0.652588229906029</v>
+        <v>0.652619594148626</v>
       </c>
     </row>
     <row r="13">
@@ -1201,55 +1201,55 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>588.5432516906337</v>
+        <v>553.8137386601779</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1910400390625</v>
+        <v>0.3394951820373535</v>
       </c>
       <c r="E13" t="n">
-        <v>173</v>
+        <v>194</v>
       </c>
       <c r="F13" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G13" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="H13" t="n">
-        <v>1367.264634466625</v>
+        <v>1256.781901355151</v>
       </c>
       <c r="I13" t="n">
-        <v>0.8242640495300293</v>
+        <v>3.959548950195312</v>
       </c>
       <c r="J13" t="n">
-        <v>220</v>
+        <v>202</v>
       </c>
       <c r="K13" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="L13" t="n">
-        <v>260</v>
+        <v>288</v>
       </c>
       <c r="M13" t="n">
-        <v>3801.963649210463</v>
+        <v>3759.205452111808</v>
       </c>
       <c r="N13" t="n">
-        <v>4.564842939376831</v>
+        <v>7.06955885887146</v>
       </c>
       <c r="O13" t="n">
-        <v>1151</v>
+        <v>1278</v>
       </c>
       <c r="P13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q13" t="n">
-        <v>3861</v>
+        <v>4293</v>
       </c>
       <c r="R13" t="n">
-        <v>0.8452001896933303</v>
+        <v>0.8526779805692551</v>
       </c>
       <c r="S13" t="n">
-        <v>0.6403793511412033</v>
+        <v>0.6656788469358256</v>
       </c>
     </row>
     <row r="14">
@@ -1262,55 +1262,55 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>577.0295752663707</v>
+        <v>565.8109130899079</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1797456741333008</v>
+        <v>0.6014730930328369</v>
       </c>
       <c r="E14" t="n">
-        <v>163</v>
+        <v>192</v>
       </c>
       <c r="F14" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="G14" t="n">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="H14" t="n">
-        <v>1167.969516485709</v>
+        <v>1174.557854368405</v>
       </c>
       <c r="I14" t="n">
-        <v>0.650580883026123</v>
+        <v>5.762675046920776</v>
       </c>
       <c r="J14" t="n">
-        <v>204</v>
+        <v>217</v>
       </c>
       <c r="K14" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="L14" t="n">
-        <v>235</v>
+        <v>302</v>
       </c>
       <c r="M14" t="n">
-        <v>3769.430160232943</v>
+        <v>3709.665506799755</v>
       </c>
       <c r="N14" t="n">
-        <v>5.231592178344727</v>
+        <v>5.789358139038086</v>
       </c>
       <c r="O14" t="n">
-        <v>1169</v>
+        <v>1275</v>
       </c>
       <c r="P14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="Q14" t="n">
-        <v>3958</v>
+        <v>4203</v>
       </c>
       <c r="R14" t="n">
-        <v>0.8469186187997415</v>
+        <v>0.8474765684257015</v>
       </c>
       <c r="S14" t="n">
-        <v>0.6901469275627776</v>
+        <v>0.6833790399119652</v>
       </c>
     </row>
     <row r="15">
@@ -1323,55 +1323,55 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>588.3329308857302</v>
+        <v>594.8873988210141</v>
       </c>
       <c r="D15" t="n">
-        <v>0.2132208347320557</v>
+        <v>0.3882570266723633</v>
       </c>
       <c r="E15" t="n">
-        <v>194</v>
+        <v>162</v>
       </c>
       <c r="F15" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="G15" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H15" t="n">
-        <v>1152.508021100977</v>
+        <v>1262.828725543841</v>
       </c>
       <c r="I15" t="n">
-        <v>0.6266262531280518</v>
+        <v>5.287035226821899</v>
       </c>
       <c r="J15" t="n">
-        <v>199</v>
+        <v>225</v>
       </c>
       <c r="K15" t="n">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="L15" t="n">
-        <v>237</v>
+        <v>310</v>
       </c>
       <c r="M15" t="n">
-        <v>3839.36036787705</v>
+        <v>3683.274910122118</v>
       </c>
       <c r="N15" t="n">
-        <v>4.707929134368896</v>
+        <v>6.768457174301147</v>
       </c>
       <c r="O15" t="n">
-        <v>1209</v>
+        <v>1259</v>
       </c>
       <c r="P15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q15" t="n">
-        <v>3983</v>
+        <v>4142</v>
       </c>
       <c r="R15" t="n">
-        <v>0.846762774391234</v>
+        <v>0.8384895471184662</v>
       </c>
       <c r="S15" t="n">
-        <v>0.699817701213015</v>
+        <v>0.6571451340562652</v>
       </c>
     </row>
     <row r="16">
@@ -1384,55 +1384,55 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>618.3579867921392</v>
+        <v>600.9734967168821</v>
       </c>
       <c r="D16" t="n">
-        <v>0.2343058586120605</v>
+        <v>0.4479141235351562</v>
       </c>
       <c r="E16" t="n">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F16" t="n">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="G16" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="H16" t="n">
-        <v>1264.953002794771</v>
+        <v>1216.06924865487</v>
       </c>
       <c r="I16" t="n">
-        <v>0.7883620262145996</v>
+        <v>4.494848012924194</v>
       </c>
       <c r="J16" t="n">
         <v>226</v>
       </c>
       <c r="K16" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="L16" t="n">
-        <v>261</v>
+        <v>306</v>
       </c>
       <c r="M16" t="n">
-        <v>3885.942131051863</v>
+        <v>3707.722039461181</v>
       </c>
       <c r="N16" t="n">
-        <v>4.932055950164795</v>
+        <v>5.850858926773071</v>
       </c>
       <c r="O16" t="n">
-        <v>1184</v>
+        <v>1250</v>
       </c>
       <c r="P16" t="n">
         <v>1</v>
       </c>
       <c r="Q16" t="n">
-        <v>3869</v>
+        <v>4078</v>
       </c>
       <c r="R16" t="n">
-        <v>0.8408730840711826</v>
+        <v>0.8379130122698687</v>
       </c>
       <c r="S16" t="n">
-        <v>0.6744797117057511</v>
+        <v>0.6720171480730542</v>
       </c>
     </row>
     <row r="17">
@@ -1445,55 +1445,55 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>557.0880873813948</v>
+        <v>601.0377204741194</v>
       </c>
       <c r="D17" t="n">
-        <v>0.2106971740722656</v>
+        <v>0.3395979404449463</v>
       </c>
       <c r="E17" t="n">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="F17" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G17" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="H17" t="n">
-        <v>1269.470079361921</v>
+        <v>1349.564249723196</v>
       </c>
       <c r="I17" t="n">
-        <v>0.6922652721405029</v>
+        <v>4.715970993041992</v>
       </c>
       <c r="J17" t="n">
-        <v>209</v>
+        <v>240</v>
       </c>
       <c r="K17" t="n">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="L17" t="n">
-        <v>251</v>
+        <v>321</v>
       </c>
       <c r="M17" t="n">
-        <v>3825.663970814586</v>
+        <v>3719.884696715515</v>
       </c>
       <c r="N17" t="n">
-        <v>4.969393730163574</v>
+        <v>5.267759084701538</v>
       </c>
       <c r="O17" t="n">
-        <v>1126</v>
+        <v>1272</v>
       </c>
       <c r="P17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>3753</v>
+        <v>4163</v>
       </c>
       <c r="R17" t="n">
-        <v>0.8543813331146343</v>
+        <v>0.8384257122257559</v>
       </c>
       <c r="S17" t="n">
-        <v>0.6681699989736378</v>
+        <v>0.6372026662775869</v>
       </c>
     </row>
     <row r="18">
@@ -1506,55 +1506,55 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>633.5644914937917</v>
+        <v>485.299621389757</v>
       </c>
       <c r="D18" t="n">
-        <v>0.2165720462799072</v>
+        <v>0.326214075088501</v>
       </c>
       <c r="E18" t="n">
-        <v>158</v>
+        <v>188</v>
       </c>
       <c r="F18" t="n">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="G18" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="H18" t="n">
-        <v>1236.570071751985</v>
+        <v>1208.087989212456</v>
       </c>
       <c r="I18" t="n">
-        <v>0.7610909938812256</v>
+        <v>4.7010338306427</v>
       </c>
       <c r="J18" t="n">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="K18" t="n">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="L18" t="n">
-        <v>255</v>
+        <v>307</v>
       </c>
       <c r="M18" t="n">
-        <v>3812.699266135572</v>
+        <v>3756.449785570055</v>
       </c>
       <c r="N18" t="n">
-        <v>4.959379196166992</v>
+        <v>5.044541120529175</v>
       </c>
       <c r="O18" t="n">
-        <v>1125</v>
+        <v>1265</v>
       </c>
       <c r="P18" t="n">
         <v>1</v>
       </c>
       <c r="Q18" t="n">
-        <v>3731</v>
+        <v>4134</v>
       </c>
       <c r="R18" t="n">
-        <v>0.8338278350141285</v>
+        <v>0.8708089688157216</v>
       </c>
       <c r="S18" t="n">
-        <v>0.6756707032376743</v>
+        <v>0.6783963427773801</v>
       </c>
     </row>
     <row r="19">
@@ -1567,55 +1567,55 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>559.5497345364762</v>
+        <v>587.6337104701369</v>
       </c>
       <c r="D19" t="n">
-        <v>0.2693681716918945</v>
+        <v>0.4412310123443604</v>
       </c>
       <c r="E19" t="n">
-        <v>202</v>
+        <v>179</v>
       </c>
       <c r="F19" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G19" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="H19" t="n">
-        <v>1316.989661275501</v>
+        <v>1235.824684562609</v>
       </c>
       <c r="I19" t="n">
-        <v>0.9265859127044678</v>
+        <v>4.921075820922852</v>
       </c>
       <c r="J19" t="n">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="K19" t="n">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="L19" t="n">
-        <v>259</v>
+        <v>297</v>
       </c>
       <c r="M19" t="n">
-        <v>3761.567609799742</v>
+        <v>3729.12397292695</v>
       </c>
       <c r="N19" t="n">
-        <v>4.879021167755127</v>
+        <v>5.873302221298218</v>
       </c>
       <c r="O19" t="n">
-        <v>1177</v>
+        <v>1277</v>
       </c>
       <c r="P19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q19" t="n">
-        <v>3945</v>
+        <v>4231</v>
       </c>
       <c r="R19" t="n">
-        <v>0.851245599553037</v>
+        <v>0.8424204411716274</v>
       </c>
       <c r="S19" t="n">
-        <v>0.6498827622174218</v>
+        <v>0.6686018771339953</v>
       </c>
     </row>
     <row r="20">
@@ -1628,55 +1628,55 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>585.8626055554621</v>
+        <v>553.0451129486112</v>
       </c>
       <c r="D20" t="n">
-        <v>0.2007732391357422</v>
+        <v>0.6170749664306641</v>
       </c>
       <c r="E20" t="n">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="F20" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G20" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H20" t="n">
-        <v>1201.718234641037</v>
+        <v>1286.459113439842</v>
       </c>
       <c r="I20" t="n">
-        <v>1.159993886947632</v>
+        <v>6.261260032653809</v>
       </c>
       <c r="J20" t="n">
-        <v>200</v>
+        <v>230</v>
       </c>
       <c r="K20" t="n">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="L20" t="n">
-        <v>242</v>
+        <v>318</v>
       </c>
       <c r="M20" t="n">
-        <v>3714.146063069804</v>
+        <v>3688.695972219228</v>
       </c>
       <c r="N20" t="n">
-        <v>4.936125993728638</v>
+        <v>5.786432981491089</v>
       </c>
       <c r="O20" t="n">
-        <v>1166</v>
+        <v>1293</v>
       </c>
       <c r="P20" t="n">
         <v>2</v>
       </c>
       <c r="Q20" t="n">
-        <v>3980</v>
+        <v>4252</v>
       </c>
       <c r="R20" t="n">
-        <v>0.8422618293392486</v>
+        <v>0.8500702912048664</v>
       </c>
       <c r="S20" t="n">
-        <v>0.676448310261714</v>
+        <v>0.6512428448620909</v>
       </c>
     </row>
     <row r="21">
@@ -1689,55 +1689,55 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>637.8434371430614</v>
+        <v>612.4559467084441</v>
       </c>
       <c r="D21" t="n">
-        <v>0.2450990676879883</v>
+        <v>0.8623459339141846</v>
       </c>
       <c r="E21" t="n">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="F21" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="G21" t="n">
+        <v>42</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1224.834508352634</v>
+      </c>
+      <c r="I21" t="n">
+        <v>4.422016859054565</v>
+      </c>
+      <c r="J21" t="n">
+        <v>225</v>
+      </c>
+      <c r="K21" t="n">
         <v>33</v>
       </c>
-      <c r="H21" t="n">
-        <v>1260.245721897462</v>
-      </c>
-      <c r="I21" t="n">
-        <v>0.7429730892181396</v>
-      </c>
-      <c r="J21" t="n">
-        <v>239</v>
-      </c>
-      <c r="K21" t="n">
-        <v>26</v>
-      </c>
       <c r="L21" t="n">
-        <v>264</v>
+        <v>306</v>
       </c>
       <c r="M21" t="n">
-        <v>3706.519056360657</v>
+        <v>3852.518814930119</v>
       </c>
       <c r="N21" t="n">
-        <v>5.128605842590332</v>
+        <v>5.947768926620483</v>
       </c>
       <c r="O21" t="n">
-        <v>1146</v>
+        <v>1279</v>
       </c>
       <c r="P21" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q21" t="n">
-        <v>3877</v>
+        <v>4166</v>
       </c>
       <c r="R21" t="n">
-        <v>0.8279130830182904</v>
+        <v>0.8410245410522276</v>
       </c>
       <c r="S21" t="n">
-        <v>0.6599921104587907</v>
+        <v>0.6820691689795547</v>
       </c>
     </row>
     <row r="22">
@@ -1750,13 +1750,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>612.3891815870101</v>
+        <v>588.0972839858694</v>
       </c>
       <c r="D22" t="n">
-        <v>0.3011198043823242</v>
+        <v>0.5386049747467041</v>
       </c>
       <c r="E22" t="n">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="F22" t="n">
         <v>30</v>
@@ -1765,40 +1765,40 @@
         <v>34</v>
       </c>
       <c r="H22" t="n">
-        <v>1182.15733015462</v>
+        <v>1248.678642776034</v>
       </c>
       <c r="I22" t="n">
-        <v>1.074103116989136</v>
+        <v>4.429054021835327</v>
       </c>
       <c r="J22" t="n">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="K22" t="n">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="L22" t="n">
-        <v>250</v>
+        <v>316</v>
       </c>
       <c r="M22" t="n">
-        <v>3889.66214032175</v>
+        <v>3779.74008610459</v>
       </c>
       <c r="N22" t="n">
-        <v>4.905173063278198</v>
+        <v>5.244836091995239</v>
       </c>
       <c r="O22" t="n">
-        <v>1127</v>
+        <v>1282</v>
       </c>
       <c r="P22" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>3760</v>
+        <v>4392</v>
       </c>
       <c r="R22" t="n">
-        <v>0.8425598009557833</v>
+        <v>0.8444080093898828</v>
       </c>
       <c r="S22" t="n">
-        <v>0.6960771173671055</v>
+        <v>0.6696390189985456</v>
       </c>
     </row>
     <row r="23">
@@ -1811,55 +1811,55 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>561.9886423054664</v>
+        <v>591.1705007329532</v>
       </c>
       <c r="D23" t="n">
-        <v>0.1932070255279541</v>
+        <v>0.3268930912017822</v>
       </c>
       <c r="E23" t="n">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="F23" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="G23" t="n">
         <v>29</v>
       </c>
       <c r="H23" t="n">
-        <v>1295.172462041263</v>
+        <v>1210.550169987005</v>
       </c>
       <c r="I23" t="n">
-        <v>0.8708410263061523</v>
+        <v>4.035156011581421</v>
       </c>
       <c r="J23" t="n">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="K23" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="L23" t="n">
-        <v>265</v>
+        <v>294</v>
       </c>
       <c r="M23" t="n">
-        <v>3820.782752421321</v>
+        <v>3667.860453770886</v>
       </c>
       <c r="N23" t="n">
-        <v>5.0416419506073</v>
+        <v>5.603813171386719</v>
       </c>
       <c r="O23" t="n">
-        <v>1183</v>
+        <v>1260</v>
       </c>
       <c r="P23" t="n">
         <v>2</v>
       </c>
       <c r="Q23" t="n">
-        <v>3858</v>
+        <v>4181</v>
       </c>
       <c r="R23" t="n">
-        <v>0.8529126938846966</v>
+        <v>0.8388241569754439</v>
       </c>
       <c r="S23" t="n">
-        <v>0.6610190775121979</v>
+        <v>0.6699574083462058</v>
       </c>
     </row>
     <row r="24">
@@ -1872,55 +1872,55 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>524.7545885914702</v>
+        <v>623.4273518702354</v>
       </c>
       <c r="D24" t="n">
-        <v>0.2083389759063721</v>
+        <v>0.3551678657531738</v>
       </c>
       <c r="E24" t="n">
-        <v>195</v>
+        <v>159</v>
       </c>
       <c r="F24" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="G24" t="n">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H24" t="n">
-        <v>1220.554262731809</v>
+        <v>1261.686808217863</v>
       </c>
       <c r="I24" t="n">
-        <v>0.7069330215454102</v>
+        <v>5.797652006149292</v>
       </c>
       <c r="J24" t="n">
         <v>226</v>
       </c>
       <c r="K24" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="L24" t="n">
-        <v>259</v>
+        <v>311</v>
       </c>
       <c r="M24" t="n">
-        <v>3755.92990507093</v>
+        <v>3782.384961475486</v>
       </c>
       <c r="N24" t="n">
-        <v>4.709434032440186</v>
+        <v>5.055239915847778</v>
       </c>
       <c r="O24" t="n">
-        <v>1152</v>
+        <v>1283</v>
       </c>
       <c r="P24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q24" t="n">
-        <v>3769</v>
+        <v>4244</v>
       </c>
       <c r="R24" t="n">
-        <v>0.8602863733204946</v>
+        <v>0.8351761234723607</v>
       </c>
       <c r="S24" t="n">
-        <v>0.6750327366109993</v>
+        <v>0.6664308839347526</v>
       </c>
     </row>
     <row r="25">
@@ -1933,55 +1933,55 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>649.6989085490291</v>
+        <v>576.5469587880644</v>
       </c>
       <c r="D25" t="n">
-        <v>0.1859159469604492</v>
+        <v>0.4718508720397949</v>
       </c>
       <c r="E25" t="n">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="F25" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G25" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="H25" t="n">
-        <v>1242.127490286532</v>
+        <v>1239.993820730697</v>
       </c>
       <c r="I25" t="n">
-        <v>0.7268538475036621</v>
+        <v>4.128710985183716</v>
       </c>
       <c r="J25" t="n">
-        <v>238</v>
+        <v>215</v>
       </c>
       <c r="K25" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="L25" t="n">
-        <v>267</v>
+        <v>306</v>
       </c>
       <c r="M25" t="n">
-        <v>3790.669010589556</v>
+        <v>3690.181334068177</v>
       </c>
       <c r="N25" t="n">
-        <v>3.816943168640137</v>
+        <v>5.295761108398438</v>
       </c>
       <c r="O25" t="n">
-        <v>1154</v>
+        <v>1257</v>
       </c>
       <c r="P25" t="n">
         <v>1</v>
       </c>
       <c r="Q25" t="n">
-        <v>3902</v>
+        <v>4161</v>
       </c>
       <c r="R25" t="n">
-        <v>0.8286057403761605</v>
+        <v>0.8437618895675081</v>
       </c>
       <c r="S25" t="n">
-        <v>0.6723197180190242</v>
+        <v>0.663974827122198</v>
       </c>
     </row>
     <row r="26">
@@ -1994,55 +1994,55 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>583.8469630141644</v>
+        <v>575.0046329536871</v>
       </c>
       <c r="D26" t="n">
-        <v>0.201563835144043</v>
+        <v>0.6647429466247559</v>
       </c>
       <c r="E26" t="n">
-        <v>169</v>
+        <v>184</v>
       </c>
       <c r="F26" t="n">
         <v>31</v>
       </c>
       <c r="G26" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="H26" t="n">
-        <v>1208.204689405017</v>
+        <v>1114.115914063393</v>
       </c>
       <c r="I26" t="n">
-        <v>0.7606830596923828</v>
+        <v>3.888550996780396</v>
       </c>
       <c r="J26" t="n">
-        <v>223</v>
+        <v>195</v>
       </c>
       <c r="K26" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="L26" t="n">
-        <v>260</v>
+        <v>269</v>
       </c>
       <c r="M26" t="n">
-        <v>3849.940542465443</v>
+        <v>3733.747927061901</v>
       </c>
       <c r="N26" t="n">
-        <v>5.139503955841064</v>
+        <v>6.692054986953735</v>
       </c>
       <c r="O26" t="n">
-        <v>1183</v>
+        <v>1309</v>
       </c>
       <c r="P26" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q26" t="n">
-        <v>3898</v>
+        <v>4357</v>
       </c>
       <c r="R26" t="n">
-        <v>0.8483490961550596</v>
+        <v>0.8459980041003571</v>
       </c>
       <c r="S26" t="n">
-        <v>0.6861757536049372</v>
+        <v>0.7016092313065991</v>
       </c>
     </row>
     <row r="27">
@@ -2055,55 +2055,55 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>574.8865380584252</v>
+        <v>601.5212993443024</v>
       </c>
       <c r="D27" t="n">
-        <v>0.1946151256561279</v>
+        <v>0.405200719833374</v>
       </c>
       <c r="E27" t="n">
-        <v>171</v>
+        <v>194</v>
       </c>
       <c r="F27" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="G27" t="n">
+        <v>41</v>
+      </c>
+      <c r="H27" t="n">
+        <v>1267.451206593123</v>
+      </c>
+      <c r="I27" t="n">
+        <v>5.13184118270874</v>
+      </c>
+      <c r="J27" t="n">
+        <v>224</v>
+      </c>
+      <c r="K27" t="n">
         <v>35</v>
       </c>
-      <c r="H27" t="n">
-        <v>1169.744429160519</v>
-      </c>
-      <c r="I27" t="n">
-        <v>0.6504409313201904</v>
-      </c>
-      <c r="J27" t="n">
-        <v>214</v>
-      </c>
-      <c r="K27" t="n">
-        <v>33</v>
-      </c>
       <c r="L27" t="n">
-        <v>246</v>
+        <v>314</v>
       </c>
       <c r="M27" t="n">
-        <v>3760.076860027626</v>
+        <v>3723.728028250181</v>
       </c>
       <c r="N27" t="n">
-        <v>5.126184940338135</v>
+        <v>5.956422805786133</v>
       </c>
       <c r="O27" t="n">
-        <v>1188</v>
+        <v>1284</v>
       </c>
       <c r="P27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q27" t="n">
-        <v>3919</v>
+        <v>4304</v>
       </c>
       <c r="R27" t="n">
-        <v>0.8471077694794246</v>
+        <v>0.8384626119896936</v>
       </c>
       <c r="S27" t="n">
-        <v>0.6889041174674485</v>
+        <v>0.6596284162061341</v>
       </c>
     </row>
     <row r="28">
@@ -2116,55 +2116,55 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>562.7074253913779</v>
+        <v>615.8534556660363</v>
       </c>
       <c r="D28" t="n">
-        <v>0.2855422496795654</v>
+        <v>0.6003057956695557</v>
       </c>
       <c r="E28" t="n">
-        <v>216</v>
+        <v>191</v>
       </c>
       <c r="F28" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="G28" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="H28" t="n">
-        <v>1174.986576261471</v>
+        <v>1321.983857576201</v>
       </c>
       <c r="I28" t="n">
-        <v>0.7683367729187012</v>
+        <v>6.702141046524048</v>
       </c>
       <c r="J28" t="n">
-        <v>207</v>
+        <v>255</v>
       </c>
       <c r="K28" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="L28" t="n">
-        <v>241</v>
+        <v>336</v>
       </c>
       <c r="M28" t="n">
-        <v>3774.576940263503</v>
+        <v>3764.394612137873</v>
       </c>
       <c r="N28" t="n">
-        <v>4.824006795883179</v>
+        <v>6.551737070083618</v>
       </c>
       <c r="O28" t="n">
-        <v>1134</v>
+        <v>1307</v>
       </c>
       <c r="P28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q28" t="n">
-        <v>3764</v>
+        <v>4205</v>
       </c>
       <c r="R28" t="n">
-        <v>0.8509217233356766</v>
+        <v>0.8364003992354347</v>
       </c>
       <c r="S28" t="n">
-        <v>0.6887103919573447</v>
+        <v>0.6488190017822226</v>
       </c>
     </row>
     <row r="29">
@@ -2177,55 +2177,55 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>610.7604864674776</v>
+        <v>595.9258224710518</v>
       </c>
       <c r="D29" t="n">
-        <v>0.2160251140594482</v>
+        <v>0.5727612972259521</v>
       </c>
       <c r="E29" t="n">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="F29" t="n">
+        <v>31</v>
+      </c>
+      <c r="G29" t="n">
+        <v>29</v>
+      </c>
+      <c r="H29" t="n">
+        <v>1276.869723237915</v>
+      </c>
+      <c r="I29" t="n">
+        <v>6.306151151657104</v>
+      </c>
+      <c r="J29" t="n">
+        <v>242</v>
+      </c>
+      <c r="K29" t="n">
         <v>33</v>
       </c>
-      <c r="G29" t="n">
-        <v>28</v>
-      </c>
-      <c r="H29" t="n">
-        <v>1216.131064394614</v>
-      </c>
-      <c r="I29" t="n">
-        <v>0.6588771343231201</v>
-      </c>
-      <c r="J29" t="n">
-        <v>206</v>
-      </c>
-      <c r="K29" t="n">
-        <v>38</v>
-      </c>
       <c r="L29" t="n">
-        <v>243</v>
+        <v>321</v>
       </c>
       <c r="M29" t="n">
-        <v>3751.64552156587</v>
+        <v>3689.2030075813</v>
       </c>
       <c r="N29" t="n">
-        <v>4.740875005722046</v>
+        <v>6.607063055038452</v>
       </c>
       <c r="O29" t="n">
-        <v>1177</v>
+        <v>1246</v>
       </c>
       <c r="P29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q29" t="n">
-        <v>3903</v>
+        <v>4179</v>
       </c>
       <c r="R29" t="n">
-        <v>0.8372019736522023</v>
+        <v>0.8384675982193374</v>
       </c>
       <c r="S29" t="n">
-        <v>0.6758406258256984</v>
+        <v>0.6538900893732461</v>
       </c>
     </row>
     <row r="30">
@@ -2238,55 +2238,55 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>545.1173472867304</v>
+        <v>559.0226052930234</v>
       </c>
       <c r="D30" t="n">
-        <v>0.2334780693054199</v>
+        <v>0.3491110801696777</v>
       </c>
       <c r="E30" t="n">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="F30" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G30" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H30" t="n">
-        <v>1218.067749475833</v>
+        <v>1186.745617807295</v>
       </c>
       <c r="I30" t="n">
-        <v>0.6455221176147461</v>
+        <v>3.748197078704834</v>
       </c>
       <c r="J30" t="n">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="K30" t="n">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="L30" t="n">
-        <v>244</v>
+        <v>268</v>
       </c>
       <c r="M30" t="n">
-        <v>3816.314313538408</v>
+        <v>3728.879442325424</v>
       </c>
       <c r="N30" t="n">
-        <v>4.28338885307312</v>
+        <v>9.511070966720581</v>
       </c>
       <c r="O30" t="n">
-        <v>1171</v>
+        <v>1296</v>
       </c>
       <c r="P30" t="n">
         <v>0</v>
       </c>
       <c r="Q30" t="n">
-        <v>3857</v>
+        <v>4272</v>
       </c>
       <c r="R30" t="n">
-        <v>0.8571613073501515</v>
+        <v>0.8500829501357109</v>
       </c>
       <c r="S30" t="n">
-        <v>0.6808261454894511</v>
+        <v>0.6817420256775021</v>
       </c>
     </row>
     <row r="31">
@@ -2299,55 +2299,55 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>589.3138668310751</v>
+        <v>664.5587469421456</v>
       </c>
       <c r="D31" t="n">
-        <v>0.1826639175415039</v>
+        <v>0.6002111434936523</v>
       </c>
       <c r="E31" t="n">
-        <v>171</v>
+        <v>190</v>
       </c>
       <c r="F31" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G31" t="n">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="H31" t="n">
-        <v>1262.423564885712</v>
+        <v>1225.149144195043</v>
       </c>
       <c r="I31" t="n">
-        <v>0.7082529067993164</v>
+        <v>5.316678762435913</v>
       </c>
       <c r="J31" t="n">
-        <v>211</v>
+        <v>234</v>
       </c>
       <c r="K31" t="n">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="L31" t="n">
-        <v>253</v>
+        <v>318</v>
       </c>
       <c r="M31" t="n">
-        <v>3754.540787741765</v>
+        <v>3706.043698428164</v>
       </c>
       <c r="N31" t="n">
-        <v>4.609005689620972</v>
+        <v>5.595330238342285</v>
       </c>
       <c r="O31" t="n">
-        <v>1131</v>
+        <v>1292</v>
       </c>
       <c r="P31" t="n">
         <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>3796</v>
+        <v>4148</v>
       </c>
       <c r="R31" t="n">
-        <v>0.8430396950926378</v>
+        <v>0.8206824309103523</v>
       </c>
       <c r="S31" t="n">
-        <v>0.6637608601809815</v>
+        <v>0.6694185919300781</v>
       </c>
     </row>
   </sheetData>

</xml_diff>